<commit_message>
fixed transform bug with text, as part of migration to jitnodes
</commit_message>
<xml_diff>
--- a/docs/project-tracker.xlsx
+++ b/docs/project-tracker.xlsx
@@ -1127,7 +1127,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G76"/>
+  <dimension ref="A1:G78"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -2375,7 +2375,7 @@
       </c>
       <c r="F37" s="19" t="inlineStr">
         <is>
-          <t>2026-10-25: GraphDock and DockController handlers go through guarded() (include/curvy/aliveguard.h) with an alive_ flag cleared in the destructor, as TimelineBar does. Removing connections instead was considered; the flag is safe whatever the view teardown order.</t>
+          <t>2026-10-25: GraphDock and DockController handlers go through guarded() (include/curvy/aliveguard.h) with an alive_ flag cleared in the destructor, as TimelineBar does. Removing connections instead was considered; the flag is safe whatever the view teardown order. Superseded 2026-10-27 by GD-07: the alive_ flag is replaced by newui::Connections.</t>
         </is>
       </c>
       <c r="G37" s="19" t="inlineStr">
@@ -3288,7 +3288,7 @@
       </c>
       <c r="D64" s="18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="E64" s="18" t="inlineStr">
@@ -3298,12 +3298,12 @@
       </c>
       <c r="F64" s="19" t="inlineStr">
         <is>
-          <t>Controllers keep a Connection per += (a Subscriptions helper) and remove them in the destructor; GraphDock/DockController/TimelineBar use alive_/guarded() meanwhile. Check newui first: if a controller cannot safely clean up (view teardown order on WM_DESTROY, or a ViewController owning its views), fix it in the framework.</t>
+          <t>2026-10-27: newui::Connections (3rdparty/newui/include/newui/delegate.h, 5 tests in unittests/test_delegate.cpp) holds the Connection of every handler and removes them in its destructor. DockController, GraphDock and TimelineBar each own one; alive_, guarded() and aliveguard.h are gone. WorkspaceController hooks frame_.onDestroyed (fires before the views are freed) and resets timeline_, graph_ and dock_ there, so their destructors only ever touch live delegates. The rule: an observer is destroyed before the subjects it observes. A liveness-token Delegate and a Subscriptions helper were rejected: a Connection removed from a dead delegate is a lifetime bug, not something to paper over. Still open: WorkspaceController's own += lambdas (GD-10).</t>
         </is>
       </c>
       <c r="G64" s="19" t="inlineStr">
         <is>
-          <t>Decided 2026-10-25; not started</t>
+          <t>Built + tested; 335 curvyTests, newui Delegate/Connections 32, checks pass; GUI suite 55 pass 2026-10-27 incl. Closing tests (T-08) exit with code 0 after Alt+F4 with all docks open; not closed by hand</t>
         </is>
       </c>
     </row>
@@ -3748,6 +3748,80 @@
       <c r="G76" s="19" t="inlineStr">
         <is>
           <t>GUI 48 pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="18" t="inlineStr">
+        <is>
+          <t>GD-10</t>
+        </is>
+      </c>
+      <c r="B77" s="18" t="inlineStr">
+        <is>
+          <t>Graph dock &amp; panels</t>
+        </is>
+      </c>
+      <c r="C77" s="19" t="inlineStr">
+        <is>
+          <t>WorkspaceController's own += lambdas that capture this (StylePanel gradient handlers, canvas onGradientStopSelected, root onKeyDown) use newui::Connections</t>
+        </is>
+      </c>
+      <c r="D77" s="18" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="E77" s="18" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="F77" s="19" t="inlineStr">
+        <is>
+          <t>Found 2026-10-27 while doing GD-07: the same hazard class as GD-04, left out because it is outside the three docks. The docks are now reset on frame_.onDestroyed, so these lambdas must tolerate a null dock_ (onGradientStopSelected already does).</t>
+        </is>
+      </c>
+      <c r="G77" s="19" t="inlineStr">
+        <is>
+          <t>Found by reading the code; not reproduced</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="18" t="inlineStr">
+        <is>
+          <t>T-08</t>
+        </is>
+      </c>
+      <c r="B78" s="18" t="inlineStr">
+        <is>
+          <t>Testing</t>
+        </is>
+      </c>
+      <c r="C78" s="19" t="inlineStr">
+        <is>
+          <t>GUI tests for closing the window and for Reset on a turned text</t>
+        </is>
+      </c>
+      <c r="D78" s="18" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E78" s="18" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F78" s="19" t="inlineStr">
+        <is>
+          <t>2026-10-27: Closing class (tests/gui/test_curvy_gui.py): Alt+F4 with toolbar, property and graph docks open, for an unmodified document and for a modified one (save question answered with N); asserts the process exit code is 0, so a teardown crash fails it. GraphDock test: a text with an off-centre pivot and 30 degrees rotation, Reset puts bounds, rotation and shear back (covers the frame-angle fix). graphdock.cpp names the Reset button graphResetButton so the driver can click it. Checked 2026-10-27 by reverting the setFrameAngle line in documentlive.cpp: the bounds alone still passed, so the test also reads transformAngleField (30 after the turn, 0 after Reset), and with the line reverted it fails at the first check. Not checked: closing by the window's X button.</t>
+        </is>
+      </c>
+      <c r="G78" s="19" t="inlineStr">
+        <is>
+          <t>Built + tested; full GUI suite 55 pass (2026-10-27), Reset test shown to fail with the fix reverted</t>
         </is>
       </c>
     </row>
@@ -3864,7 +3938,7 @@
     <row r="11">
       <c r="A11" s="19" t="inlineStr">
         <is>
-          <t>Test counts at snapshot time (2026-10-27): curvyTests 335 pass (1 skipped); GUI suite 52 (48 + 4 new; only the 11 GraphDock tests rerun); jitnodesTests 98 at 2026-10-25, not rerun; --check, --check-tools, --check-workspace exit 0. These are typed-in numbers, not formulas.</t>
+          <t>Test counts at snapshot time (2026-10-27): curvyTests 335 pass (1 skipped); GUI suite 55 pass (full run 2026-10-27); jitnodesTests 98 at 2026-10-25, not rerun; newui Delegate + Connections tests 32 pass (2026-10-27); --check, --check-tools, --check-workspace exit 0. These are typed-in numbers, not formulas.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
hitesting, new node setup,
</commit_message>
<xml_diff>
--- a/docs/project-tracker.xlsx
+++ b/docs/project-tracker.xlsx
@@ -1542,12 +1542,12 @@
       </c>
       <c r="F12" s="19" t="inlineStr">
         <is>
-          <t>Step 3/4 of the node-architecture plan. 2026-10-28: S0 spike done -&gt; option B (structure nodes in the flat root); DG-07 later removed the subnet undo cost, so option A is open again if wanted. 2026-10-28: option A (containment) chosen. S1 done: NodeRef{scope,id}, GraphDocument scopes/NodeRef edit API, SketchObject::graphScope; root-scope NodeId shortcuts kept; callers move to NodeRef in S2/S3. S2 done 2026-10-28: curvySubnet node (role/visible/locked/opacity/blend/clip + promoted placement numbers), SketchDocument::scopeMatrix/worldOf/transformRefOf, sync loops and caches per scope (a hand-built group moves its member, undo/redo works); transformNodeOf/selection/graph dock still root-only until S3/S5. Next: S3 groups by containment. Plan: docs/dg04-layers-subnets.md. Idea logged: packed-paths node (Houdini packed geometry).</t>
+          <t>Step 3/4 of the node-architecture plan. 2026-10-28: S0 spike done -&gt; option B (structure nodes in the flat root); DG-07 later removed the subnet undo cost, so option A is open again if wanted. 2026-10-28: option A (containment) chosen. S1 done: NodeRef{scope,id}, GraphDocument scopes/NodeRef edit API, SketchObject::graphScope; root-scope NodeId shortcuts kept; callers move to NodeRef in S2/S3. S2 done 2026-10-28: curvySubnet node (role/visible/locked/opacity/blend/clip + promoted placement numbers), SketchDocument::scopeMatrix/worldOf/transformRefOf, sync loops and caches per scope (a hand-built group moves its member, undo/redo works); transformNodeOf/selection/graph dock still root-only until S3/S5. S2.5 done 2026-10-28: membership accessors on SketchDocument (groupsOf/outermostGroupOf/isGrouped/inGroup/layerOf/setGroupsOf/setLayerOf) in front of SketchObject::groups()/layer(); all production sites outside the serializers (writeObject, SVG readers, sketchbin) use them. S3a done 2026-10-28: groups are real subnets by containment, derived from the group ids (syncGroupScopes/pruneGroupScopes in changed(), curvySubnet groupId param; chains copied so expressions/keys survive; SVG data-graph-scope and .skb scope paths). S5 (scoped selection) done 2026-10-28: hitTestNode/selectedNodes/setSelectedNodes return NodeRef, pivot code and the graph dock (rows, detail box, links, edits) work on NodeRef so grouped objects show and edit; enter/exit-group view not built. Next: S3b flip the carrier (drop groups_/groupProps_, read from subnets). Plan: docs/dg04-layers-subnets.md. Idea logged: packed-paths node (Houdini packed geometry).</t>
         </is>
       </c>
       <c r="G12" s="19" t="inlineStr">
         <is>
-          <t>S2 built + tested: 2082 ctest pass, --check/--check-tools/--check-workspace exit 0; GUI suite not rerun</t>
+          <t>S5 built + tested: new test NodeSelection.GroupedObjectsAreSelectedAndPickedByTheirScopedNode; ctest 2086 pass, --check/--check-tools/--check-workspace exit 0; GUI suite not rerun</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
hitesting, new node setup, groups
</commit_message>
<xml_diff>
--- a/docs/project-tracker.xlsx
+++ b/docs/project-tracker.xlsx
@@ -1542,12 +1542,12 @@
       </c>
       <c r="F12" s="19" t="inlineStr">
         <is>
-          <t>Step 3/4 of the node-architecture plan. 2026-10-28: S0 spike done -&gt; option B (structure nodes in the flat root); DG-07 later removed the subnet undo cost, so option A is open again if wanted. 2026-10-28: option A (containment) chosen. S1 done: NodeRef{scope,id}, GraphDocument scopes/NodeRef edit API, SketchObject::graphScope; root-scope NodeId shortcuts kept; callers move to NodeRef in S2/S3. S2 done 2026-10-28: curvySubnet node (role/visible/locked/opacity/blend/clip + promoted placement numbers), SketchDocument::scopeMatrix/worldOf/transformRefOf, sync loops and caches per scope (a hand-built group moves its member, undo/redo works); transformNodeOf/selection/graph dock still root-only until S3/S5. S2.5 done 2026-10-28: membership accessors on SketchDocument (groupsOf/outermostGroupOf/isGrouped/inGroup/layerOf/setGroupsOf/setLayerOf) in front of SketchObject::groups()/layer(); all production sites outside the serializers (writeObject, SVG readers, sketchbin) use them. S3a done 2026-10-28: groups are real subnets by containment, derived from the group ids (syncGroupScopes/pruneGroupScopes in changed(), curvySubnet groupId param; chains copied so expressions/keys survive; SVG data-graph-scope and .skb scope paths). S5 (scoped selection) done 2026-10-28: hitTestNode/selectedNodes/setSelectedNodes return NodeRef, pivot code and the graph dock (rows, detail box, links, edits) work on NodeRef so grouped objects show and edit; enter/exit-group view not built. Next: S3b flip the carrier (drop groups_/groupProps_, read from subnets). Plan: docs/dg04-layers-subnets.md. Idea logged: packed-paths node (Houdini packed geometry).</t>
+          <t>Step 3/4 of the node-architecture plan. 2026-10-28: S0 spike done -&gt; option B (structure nodes in the flat root); DG-07 later removed the subnet undo cost, so option A is open again if wanted. 2026-10-28: option A (containment) chosen. S1 done: NodeRef{scope,id}, GraphDocument scopes/NodeRef edit API, SketchObject::graphScope; root-scope NodeId shortcuts kept; callers move to NodeRef in S2/S3. S2 done 2026-10-28: curvySubnet node (role/visible/locked/opacity/blend/clip + promoted placement numbers), SketchDocument::scopeMatrix/worldOf/transformRefOf, sync loops and caches per scope (a hand-built group moves its member, undo/redo works); transformNodeOf/selection/graph dock still root-only until S3/S5. S2.5 done 2026-10-28: membership accessors on SketchDocument (groupsOf/outermostGroupOf/isGrouped/inGroup/layerOf/setGroupsOf/setLayerOf) in front of SketchObject::groups()/layer(); all production sites outside the serializers (writeObject, SVG readers, sketchbin) use them. S3a done 2026-10-28: groups are real subnets by containment, derived from the group ids (syncGroupScopes/pruneGroupScopes in changed(), curvySubnet groupId param; chains copied so expressions/keys survive; SVG data-graph-scope and .skb scope paths). S5 (scoped selection) done 2026-10-28: hitTestNode/selectedNodes/setSelectedNodes return NodeRef, pivot code and the graph dock (rows, detail box, links, edits) work on NodeRef so grouped objects show and edit; enter/exit-group view not built. S3b done 2026-10-29: the graph is now the carrier (syncGroupScopes merges: an edited groups() moves the chain, otherwise the subnet the chain sits in wins; group opacity/blend/clip live in the subnet node, groupProps_ only holds props of a group with no subnet; GraphDocument::scopeOf interns parent scopes). groups_/groupProps_ not deleted (clones/loaders have no document). Next: S4 layers by containment, enter/exit-group view, rerun GUI suite. Plan: docs/dg04-layers-subnets.md. Idea logged: packed-paths node (Houdini packed geometry).</t>
         </is>
       </c>
       <c r="G12" s="19" t="inlineStr">
         <is>
-          <t>S5 built + tested: new test NodeSelection.GroupedObjectsAreSelectedAndPickedByTheirScopedNode; ctest 2086 pass, --check/--check-tools/--check-workspace exit 0; GUI suite not rerun</t>
+          <t>S3b built + tested: new test SketchDocumentScopes.GroupPropsLiveInTheSubnet; ctest 2087 (ClipboardManager test flaky, passes alone), --check/--check-tools/--check-workspace exit 0; GUI suite not rerun</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
more node migration work especially to allow for layers and groups as subnets
</commit_message>
<xml_diff>
--- a/docs/project-tracker.xlsx
+++ b/docs/project-tracker.xlsx
@@ -1542,12 +1542,12 @@
       </c>
       <c r="F12" s="19" t="inlineStr">
         <is>
-          <t>Step 3/4 of the node-architecture plan. 2026-10-28: S0 spike done -&gt; option B (structure nodes in the flat root); DG-07 later removed the subnet undo cost, so option A is open again if wanted. 2026-10-28: option A (containment) chosen. S1 done: NodeRef{scope,id}, GraphDocument scopes/NodeRef edit API, SketchObject::graphScope; root-scope NodeId shortcuts kept; callers move to NodeRef in S2/S3. S2 done 2026-10-28: curvySubnet node (role/visible/locked/opacity/blend/clip + promoted placement numbers), SketchDocument::scopeMatrix/worldOf/transformRefOf, sync loops and caches per scope (a hand-built group moves its member, undo/redo works); transformNodeOf/selection/graph dock still root-only until S3/S5. S2.5 done 2026-10-28: membership accessors on SketchDocument (groupsOf/outermostGroupOf/isGrouped/inGroup/layerOf/setGroupsOf/setLayerOf) in front of SketchObject::groups()/layer(); all production sites outside the serializers (writeObject, SVG readers, sketchbin) use them. S3a done 2026-10-28: groups are real subnets by containment, derived from the group ids (syncGroupScopes/pruneGroupScopes in changed(), curvySubnet groupId param; chains copied so expressions/keys survive; SVG data-graph-scope and .skb scope paths). S5 (scoped selection) done 2026-10-28: hitTestNode/selectedNodes/setSelectedNodes return NodeRef, pivot code and the graph dock (rows, detail box, links, edits) work on NodeRef so grouped objects show and edit; enter/exit-group view not built. S3b done 2026-10-29: the graph is now the carrier (syncGroupScopes merges: an edited groups() moves the chain, otherwise the subnet the chain sits in wins; group opacity/blend/clip live in the subnet node, groupProps_ only holds props of a group with no subnet; GraphDocument::scopeOf interns parent scopes). groups_/groupProps_ not deleted (clones/loaders have no document). Next: S4 layers by containment, enter/exit-group view, rerun GUI suite. Plan: docs/dg04-layers-subnets.md. Idea logged: packed-paths node (Houdini packed geometry).</t>
+          <t>Step 3/4 of the node-architecture plan. 2026-10-28: S0 spike done -&gt; option B (structure nodes in the flat root); DG-07 later removed the subnet undo cost, so option A is open again if wanted. 2026-10-28: option A (containment) chosen. S1 done: NodeRef{scope,id}, GraphDocument scopes/NodeRef edit API, SketchObject::graphScope; root-scope NodeId shortcuts kept; callers move to NodeRef in S2/S3. S2 done 2026-10-28: curvySubnet node (role/visible/locked/opacity/blend/clip + promoted placement numbers), SketchDocument::scopeMatrix/worldOf/transformRefOf, sync loops and caches per scope (a hand-built group moves its member, undo/redo works); transformNodeOf/selection/graph dock still root-only until S3/S5. S2.5 done 2026-10-28: membership accessors on SketchDocument (groupsOf/outermostGroupOf/isGrouped/inGroup/layerOf/setGroupsOf/setLayerOf) in front of SketchObject::groups()/layer(); all production sites outside the serializers (writeObject, SVG readers, sketchbin) use them. S3a done 2026-10-28: groups are real subnets by containment, derived from the group ids (syncGroupScopes/pruneGroupScopes in changed(), curvySubnet groupId param; chains copied so expressions/keys survive; SVG data-graph-scope and .skb scope paths). S5 (scoped selection) done 2026-10-28: hitTestNode/selectedNodes/setSelectedNodes return NodeRef, pivot code and the graph dock (rows, detail box, links, edits) work on NodeRef so grouped objects show and edit; enter/exit-group view not built. S3b done 2026-10-29: the graph is now the carrier (syncGroupScopes merges: an edited groups() moves the chain, otherwise the subnet the chain sits in wins; group opacity/blend/clip live in the subnet node, groupProps_ only holds props of a group with no subnet; GraphDocument::scopeOf interns parent scopes). groups_/groupProps_ not deleted (clones/loaders have no document). S4 prerequisite 1 (partly) done 2026-10-30: tagNodeOf/addMovePoints return NodeRef, transformNodeOf removed (transformRefOf everywhere), checks and the placement/tag/key/expression tests moved to NodeRef; remaining root-only code: Flow view, GraphRow::node, the NodeId shortcuts, tests that count doc.network() nodes, .skb loader curve fix-up. Tag docs: docs/point-tags.md. S4 prereqs 2 and 3 done 2026-10-30: sync measured (linear, ~1.5 us per object per edit; the cost is object MOVES, ~0.25 ms each) so not rebuilt, test SketchDocumentScopes.AnEditCostsLittleWhenManyObjectsAreGrouped added, appearance orphan rescan skipped on a single add (~28% of path sync); default-layer decision: root holds the first top-level layer, other layers/sublayers are subnets (docs/dg04-layers-subnets.md S4). Enter/exit-group view in the graph dock built 2026-10-30 (GraphDock::viewScope/enterGroup/enterSubnet/exitGroup, Enter button, .. row, Esc; canvas does not scope). Next: S4 itself (batched migration, layer subnets, merge-node order). Plan: docs/dg04-layers-subnets.md. Idea logged: packed-paths node (Houdini packed geometry).</t>
         </is>
       </c>
       <c r="G12" s="19" t="inlineStr">
         <is>
-          <t>S3b built + tested: new test SketchDocumentScopes.GroupPropsLiveInTheSubnet; ctest 2087 (ClipboardManager test flaky, passes alone), --check/--check-tools/--check-workspace exit 0; GUI suite not rerun</t>
+          <t>Enter/exit view: build clean, curvyTests 342 pass, --check-workspace group checks pass, GUI suite 57/57 pass (2026-10-30, incl. 2 new enter/exit tests)</t>
         </is>
       </c>
     </row>
@@ -3975,7 +3975,7 @@
     <row r="11">
       <c r="A11" s="19" t="inlineStr">
         <is>
-          <t>Test counts at snapshot time (2026-10-27): curvyTests 335 pass (1 skipped); GUI suite 55 pass (full run 2026-10-27); jitnodesTests 98 at 2026-10-25, not rerun; newui Delegate + Connections tests 32 pass (2026-10-27); --check, --check-tools, --check-workspace exit 0. These are typed-in numbers, not formulas.</t>
+          <t>Test counts at snapshot time (2026-10-30): curvyTests 342 pass (1 skipped); GUI suite 57 pass (full run 2026-10-30); jitnodesTests 98 at 2026-10-25, not rerun; newui Delegate + Connections tests 32 pass (2026-10-27); --check, --check-tools, --check-workspace exit 0. These are typed-in numbers, not formulas.</t>
         </is>
       </c>
     </row>

</xml_diff>